<commit_message>
#7 Client BOM Price Edit
</commit_message>
<xml_diff>
--- a/Design Files/Xponent-tech/BOM/Client-BOM-Xponent-tech.xlsx
+++ b/Design Files/Xponent-tech/BOM/Client-BOM-Xponent-tech.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="1 Board" sheetId="1" r:id="rId1"/>
@@ -1389,15 +1389,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="17" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1410,14 +1401,6 @@
     <xf numFmtId="165" fontId="17" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="166" fontId="14" fillId="3" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1429,6 +1412,23 @@
     </xf>
     <xf numFmtId="165" fontId="17" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1904,10 +1904,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1943,7 +1943,7 @@
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="66"/>
+      <c r="L3" s="74"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1961,7 +1961,7 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="46"/>
-      <c r="L4" s="67"/>
+      <c r="L4" s="75"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1979,7 +1979,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="46"/>
-      <c r="L5" s="67"/>
+      <c r="L5" s="75"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1993,7 +1993,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="46"/>
-      <c r="L6" s="67"/>
+      <c r="L6" s="75"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2007,7 +2007,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="67"/>
+      <c r="L7" s="75"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2021,7 +2021,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="67"/>
+      <c r="L8" s="75"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2089,8 +2089,8 @@
       <c r="J10" s="27">
         <v>4</v>
       </c>
-      <c r="K10" s="68">
-        <v>1.2999999999999998</v>
+      <c r="K10" s="65">
+        <v>0.65</v>
       </c>
       <c r="L10" s="27"/>
     </row>
@@ -2124,8 +2124,8 @@
       <c r="J11" s="28">
         <v>4</v>
       </c>
-      <c r="K11" s="69">
-        <v>1.278</v>
+      <c r="K11" s="66">
+        <v>0.7</v>
       </c>
       <c r="L11" s="28"/>
     </row>
@@ -2159,8 +2159,8 @@
       <c r="J12" s="27">
         <v>1</v>
       </c>
-      <c r="K12" s="68">
-        <v>1.125</v>
+      <c r="K12" s="65">
+        <v>0.3</v>
       </c>
       <c r="L12" s="27"/>
     </row>
@@ -2194,8 +2194,8 @@
       <c r="J13" s="28">
         <v>1</v>
       </c>
-      <c r="K13" s="69">
-        <v>1</v>
+      <c r="K13" s="66">
+        <v>0.3</v>
       </c>
       <c r="L13" s="28"/>
     </row>
@@ -2229,8 +2229,8 @@
       <c r="J14" s="27">
         <v>1</v>
       </c>
-      <c r="K14" s="68">
-        <v>1.1339999999999999</v>
+      <c r="K14" s="65">
+        <v>0.3</v>
       </c>
       <c r="L14" s="27"/>
     </row>
@@ -2264,7 +2264,7 @@
       <c r="J15" s="28">
         <v>2</v>
       </c>
-      <c r="K15" s="69">
+      <c r="K15" s="66">
         <v>1.258</v>
       </c>
       <c r="L15" s="28"/>
@@ -2299,8 +2299,8 @@
       <c r="J16" s="27">
         <v>1</v>
       </c>
-      <c r="K16" s="68">
-        <v>1.1499999999999999</v>
+      <c r="K16" s="65">
+        <v>0.35</v>
       </c>
       <c r="L16" s="27"/>
     </row>
@@ -2334,8 +2334,8 @@
       <c r="J17" s="28">
         <v>1</v>
       </c>
-      <c r="K17" s="69">
-        <v>1.1599999999999999</v>
+      <c r="K17" s="66">
+        <v>0.25</v>
       </c>
       <c r="L17" s="28"/>
     </row>
@@ -2369,8 +2369,8 @@
       <c r="J18" s="27">
         <v>1</v>
       </c>
-      <c r="K18" s="68">
-        <v>1.08</v>
+      <c r="K18" s="65">
+        <v>0.25</v>
       </c>
       <c r="L18" s="27"/>
     </row>
@@ -2404,8 +2404,8 @@
       <c r="J19" s="28">
         <v>2</v>
       </c>
-      <c r="K19" s="69">
-        <v>1.9411</v>
+      <c r="K19" s="66">
+        <v>0.4</v>
       </c>
       <c r="L19" s="28"/>
     </row>
@@ -2439,8 +2439,8 @@
       <c r="J20" s="27">
         <v>1</v>
       </c>
-      <c r="K20" s="68">
-        <v>1.345</v>
+      <c r="K20" s="65">
+        <v>0.25</v>
       </c>
       <c r="L20" s="27"/>
     </row>
@@ -2474,8 +2474,8 @@
       <c r="J21" s="28">
         <v>1</v>
       </c>
-      <c r="K21" s="69">
-        <v>1.3363999999999998</v>
+      <c r="K21" s="66">
+        <v>0.3</v>
       </c>
       <c r="L21" s="28"/>
     </row>
@@ -2509,8 +2509,8 @@
       <c r="J22" s="27">
         <v>1</v>
       </c>
-      <c r="K22" s="68">
-        <v>0.95499999999999996</v>
+      <c r="K22" s="65">
+        <v>0.2</v>
       </c>
       <c r="L22" s="27"/>
     </row>
@@ -2544,8 +2544,8 @@
       <c r="J23" s="28">
         <v>1</v>
       </c>
-      <c r="K23" s="69">
-        <v>1.3919999999999999</v>
+      <c r="K23" s="66">
+        <v>0.35</v>
       </c>
       <c r="L23" s="28"/>
     </row>
@@ -2579,8 +2579,8 @@
       <c r="J24" s="27">
         <v>1</v>
       </c>
-      <c r="K24" s="68">
-        <v>1.1179999999999999</v>
+      <c r="K24" s="65">
+        <v>0.3</v>
       </c>
       <c r="L24" s="27"/>
     </row>
@@ -2614,8 +2614,8 @@
       <c r="J25" s="28">
         <v>1</v>
       </c>
-      <c r="K25" s="69">
-        <v>1.4049999999999998</v>
+      <c r="K25" s="66">
+        <v>0.35</v>
       </c>
       <c r="L25" s="28"/>
     </row>
@@ -2649,8 +2649,8 @@
       <c r="J26" s="27">
         <v>1</v>
       </c>
-      <c r="K26" s="68">
-        <v>1.0549999999999999</v>
+      <c r="K26" s="65">
+        <v>1.72</v>
       </c>
       <c r="L26" s="27"/>
     </row>
@@ -2684,8 +2684,8 @@
       <c r="J27" s="28">
         <v>2</v>
       </c>
-      <c r="K27" s="69">
-        <v>2.2290000000000001</v>
+      <c r="K27" s="66">
+        <v>2.58</v>
       </c>
       <c r="L27" s="28"/>
     </row>
@@ -2719,8 +2719,8 @@
       <c r="J28" s="27">
         <v>13</v>
       </c>
-      <c r="K28" s="68">
-        <v>1.1459999999999999</v>
+      <c r="K28" s="65">
+        <v>0.88</v>
       </c>
       <c r="L28" s="27"/>
     </row>
@@ -2754,8 +2754,8 @@
       <c r="J29" s="28">
         <v>1</v>
       </c>
-      <c r="K29" s="69">
-        <v>1.4550000000000001</v>
+      <c r="K29" s="66">
+        <v>0.72</v>
       </c>
       <c r="L29" s="28"/>
     </row>
@@ -2789,8 +2789,8 @@
       <c r="J30" s="27">
         <v>4</v>
       </c>
-      <c r="K30" s="68">
-        <v>1.1499999999999999</v>
+      <c r="K30" s="65">
+        <v>0.47</v>
       </c>
       <c r="L30" s="27"/>
     </row>
@@ -2824,8 +2824,8 @@
       <c r="J31" s="28">
         <v>2</v>
       </c>
-      <c r="K31" s="69">
-        <v>1.2999999999999998</v>
+      <c r="K31" s="66">
+        <v>0.4</v>
       </c>
       <c r="L31" s="28"/>
     </row>
@@ -2859,8 +2859,8 @@
       <c r="J32" s="27">
         <v>1</v>
       </c>
-      <c r="K32" s="68">
-        <v>1.268</v>
+      <c r="K32" s="65">
+        <v>0.25</v>
       </c>
       <c r="L32" s="27"/>
     </row>
@@ -2894,7 +2894,7 @@
       <c r="J33" s="28">
         <v>1</v>
       </c>
-      <c r="K33" s="69">
+      <c r="K33" s="66">
         <v>2.4249999999999998</v>
       </c>
       <c r="L33" s="28"/>
@@ -2929,8 +2929,8 @@
       <c r="J34" s="28">
         <v>2</v>
       </c>
-      <c r="K34" s="68">
-        <v>1.292</v>
+      <c r="K34" s="65">
+        <v>0.45</v>
       </c>
       <c r="L34" s="27"/>
     </row>
@@ -2964,8 +2964,8 @@
       <c r="J35" s="27">
         <v>1</v>
       </c>
-      <c r="K35" s="68">
-        <v>1.2439999999999998</v>
+      <c r="K35" s="65">
+        <v>0.3</v>
       </c>
       <c r="L35" s="28"/>
     </row>
@@ -2999,8 +2999,8 @@
       <c r="J36" s="28">
         <v>2</v>
       </c>
-      <c r="K36" s="68">
-        <v>1.115</v>
+      <c r="K36" s="65">
+        <v>0.38</v>
       </c>
       <c r="L36" s="27"/>
     </row>
@@ -3034,8 +3034,8 @@
       <c r="J37" s="27">
         <v>3</v>
       </c>
-      <c r="K37" s="68">
-        <v>1.1299999999999999</v>
+      <c r="K37" s="65">
+        <v>0.57999999999999996</v>
       </c>
       <c r="L37" s="28"/>
     </row>
@@ -3069,8 +3069,8 @@
       <c r="J38" s="28">
         <v>2</v>
       </c>
-      <c r="K38" s="68">
-        <v>1.202</v>
+      <c r="K38" s="65">
+        <v>0.6</v>
       </c>
       <c r="L38" s="27"/>
     </row>
@@ -3104,8 +3104,8 @@
       <c r="J39" s="27">
         <v>3</v>
       </c>
-      <c r="K39" s="68">
-        <v>1.272</v>
+      <c r="K39" s="65">
+        <v>0.7</v>
       </c>
       <c r="L39" s="28"/>
     </row>
@@ -3139,8 +3139,8 @@
       <c r="J40" s="28">
         <v>2</v>
       </c>
-      <c r="K40" s="68">
-        <v>1.1099999999999999</v>
+      <c r="K40" s="65">
+        <v>0.37</v>
       </c>
       <c r="L40" s="27"/>
     </row>
@@ -3174,8 +3174,8 @@
       <c r="J41" s="27">
         <v>3</v>
       </c>
-      <c r="K41" s="68">
-        <v>1.2959999999999998</v>
+      <c r="K41" s="65">
+        <v>0.49</v>
       </c>
       <c r="L41" s="28"/>
     </row>
@@ -3207,8 +3207,8 @@
       <c r="J42" s="28">
         <v>3</v>
       </c>
-      <c r="K42" s="68">
-        <v>0.76999999999999991</v>
+      <c r="K42" s="65">
+        <v>0.7</v>
       </c>
       <c r="L42" s="27"/>
     </row>
@@ -3242,8 +3242,8 @@
       <c r="J43" s="27">
         <v>2</v>
       </c>
-      <c r="K43" s="68">
-        <v>0.82</v>
+      <c r="K43" s="65">
+        <v>0.25</v>
       </c>
       <c r="L43" s="28"/>
     </row>
@@ -3277,8 +3277,8 @@
       <c r="J44" s="28">
         <v>3</v>
       </c>
-      <c r="K44" s="68">
-        <v>1.2439999999999998</v>
+      <c r="K44" s="65">
+        <v>0.45</v>
       </c>
       <c r="L44" s="27"/>
     </row>
@@ -3312,8 +3312,8 @@
       <c r="J45" s="27">
         <v>2</v>
       </c>
-      <c r="K45" s="68">
-        <v>1.198</v>
+      <c r="K45" s="65">
+        <v>0.36</v>
       </c>
       <c r="L45" s="28"/>
     </row>
@@ -3347,8 +3347,8 @@
       <c r="J46" s="28">
         <v>3</v>
       </c>
-      <c r="K46" s="68">
-        <v>1.3039999999999998</v>
+      <c r="K46" s="65">
+        <v>0.9</v>
       </c>
       <c r="L46" s="27"/>
     </row>
@@ -3382,8 +3382,8 @@
       <c r="J47" s="27">
         <v>2</v>
       </c>
-      <c r="K47" s="68">
-        <v>1.2559999999999998</v>
+      <c r="K47" s="65">
+        <v>0.55000000000000004</v>
       </c>
       <c r="L47" s="28"/>
     </row>
@@ -3417,8 +3417,8 @@
       <c r="J48" s="28">
         <v>2</v>
       </c>
-      <c r="K48" s="68">
-        <v>1.3479999999999999</v>
+      <c r="K48" s="65">
+        <v>0.65</v>
       </c>
       <c r="L48" s="27"/>
     </row>
@@ -3452,8 +3452,8 @@
       <c r="J49" s="27">
         <v>3</v>
       </c>
-      <c r="K49" s="68">
-        <v>1.216</v>
+      <c r="K49" s="65">
+        <v>0.85</v>
       </c>
       <c r="L49" s="28"/>
     </row>
@@ -3487,8 +3487,8 @@
       <c r="J50" s="28">
         <v>1</v>
       </c>
-      <c r="K50" s="68">
-        <v>1.2879999999999998</v>
+      <c r="K50" s="65">
+        <v>0.2</v>
       </c>
       <c r="L50" s="27"/>
     </row>
@@ -3522,8 +3522,8 @@
       <c r="J51" s="27">
         <v>1</v>
       </c>
-      <c r="K51" s="68">
-        <v>0.8899999999999999</v>
+      <c r="K51" s="65">
+        <v>0.4</v>
       </c>
       <c r="L51" s="28"/>
     </row>
@@ -3557,8 +3557,8 @@
       <c r="J52" s="28">
         <v>1</v>
       </c>
-      <c r="K52" s="68">
-        <v>1.472</v>
+      <c r="K52" s="65">
+        <v>0.3</v>
       </c>
       <c r="L52" s="27"/>
     </row>
@@ -3592,8 +3592,8 @@
       <c r="J53" s="27">
         <v>1</v>
       </c>
-      <c r="K53" s="68">
-        <v>1.1339999999999999</v>
+      <c r="K53" s="65">
+        <v>0.25</v>
       </c>
       <c r="L53" s="28"/>
     </row>
@@ -3627,8 +3627,8 @@
       <c r="J54" s="28">
         <v>1</v>
       </c>
-      <c r="K54" s="68">
-        <v>1.3239999999999998</v>
+      <c r="K54" s="65">
+        <v>0.25</v>
       </c>
       <c r="L54" s="27"/>
     </row>
@@ -3662,8 +3662,8 @@
       <c r="J55" s="27">
         <v>1</v>
       </c>
-      <c r="K55" s="68">
-        <v>1.204</v>
+      <c r="K55" s="65">
+        <v>0.25</v>
       </c>
       <c r="L55" s="28"/>
     </row>
@@ -3697,8 +3697,8 @@
       <c r="J56" s="28">
         <v>1</v>
       </c>
-      <c r="K56" s="68">
-        <v>1.1739999999999999</v>
+      <c r="K56" s="65">
+        <v>0.25</v>
       </c>
       <c r="L56" s="27"/>
     </row>
@@ -3732,8 +3732,8 @@
       <c r="J57" s="28">
         <v>1</v>
       </c>
-      <c r="K57" s="69">
-        <v>1.42</v>
+      <c r="K57" s="66">
+        <v>0.8</v>
       </c>
       <c r="L57" s="28"/>
     </row>
@@ -3767,8 +3767,8 @@
       <c r="J58" s="27">
         <v>2</v>
       </c>
-      <c r="K58" s="68">
-        <v>1.208</v>
+      <c r="K58" s="65">
+        <v>0.42</v>
       </c>
       <c r="L58" s="27"/>
     </row>
@@ -3802,7 +3802,7 @@
       <c r="J59" s="43">
         <v>2</v>
       </c>
-      <c r="K59" s="76" t="s">
+      <c r="K59" s="71" t="s">
         <v>236</v>
       </c>
       <c r="L59" s="27"/>
@@ -3837,8 +3837,8 @@
       <c r="J60" s="27">
         <v>9</v>
       </c>
-      <c r="K60" s="68">
-        <v>11.042</v>
+      <c r="K60" s="65">
+        <v>13.6</v>
       </c>
       <c r="L60" s="27"/>
     </row>
@@ -3872,8 +3872,8 @@
       <c r="J61" s="51">
         <v>3</v>
       </c>
-      <c r="K61" s="77">
-        <v>1.839</v>
+      <c r="K61" s="72">
+        <v>3.8</v>
       </c>
       <c r="L61" s="27"/>
     </row>
@@ -3884,14 +3884,14 @@
       <c r="E62" s="55"/>
       <c r="F62" s="56"/>
       <c r="G62" s="57"/>
-      <c r="H62" s="72" t="s">
+      <c r="H62" s="76" t="s">
         <v>259</v>
       </c>
-      <c r="I62" s="73"/>
-      <c r="J62" s="73"/>
-      <c r="K62" s="74">
+      <c r="I62" s="77"/>
+      <c r="J62" s="77"/>
+      <c r="K62" s="69">
         <f>SUM(K10:K61)</f>
-        <v>74.817499999999995</v>
+        <v>45.052999999999997</v>
       </c>
       <c r="L62" s="57"/>
     </row>
@@ -3935,11 +3935,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3977,7 +3977,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="66"/>
+      <c r="M3" s="74"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -3996,7 +3996,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="46"/>
       <c r="L4" s="46"/>
-      <c r="M4" s="67"/>
+      <c r="M4" s="75"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4015,7 +4015,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="46"/>
       <c r="L5" s="46"/>
-      <c r="M5" s="67"/>
+      <c r="M5" s="75"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4030,7 +4030,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="46"/>
       <c r="L6" s="46"/>
-      <c r="M6" s="67"/>
+      <c r="M6" s="75"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4045,7 +4045,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="67"/>
+      <c r="M7" s="75"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4060,7 +4060,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="67"/>
+      <c r="M8" s="75"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -4135,8 +4135,8 @@
         <f>J10*2</f>
         <v>8</v>
       </c>
-      <c r="L10" s="68">
-        <v>1.35</v>
+      <c r="L10" s="65">
+        <v>0.8</v>
       </c>
       <c r="M10" s="27"/>
     </row>
@@ -4174,8 +4174,8 @@
         <f t="shared" ref="K11:K61" si="1">J11*2</f>
         <v>8</v>
       </c>
-      <c r="L11" s="68">
-        <v>1.3279999999999998</v>
+      <c r="L11" s="66">
+        <v>0.75</v>
       </c>
       <c r="M11" s="28"/>
     </row>
@@ -4213,8 +4213,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L12" s="68">
-        <v>1.175</v>
+      <c r="L12" s="65">
+        <v>0.3</v>
       </c>
       <c r="M12" s="27"/>
     </row>
@@ -4252,8 +4252,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L13" s="68">
-        <v>1.05</v>
+      <c r="L13" s="66">
+        <v>0.3</v>
       </c>
       <c r="M13" s="28"/>
     </row>
@@ -4291,8 +4291,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L14" s="68">
-        <v>1.1839999999999999</v>
+      <c r="L14" s="65">
+        <v>0.3</v>
       </c>
       <c r="M14" s="27"/>
     </row>
@@ -4330,8 +4330,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L15" s="68">
-        <v>1.3080000000000001</v>
+      <c r="L15" s="66">
+        <v>2.4500000000000002</v>
       </c>
       <c r="M15" s="28"/>
     </row>
@@ -4369,8 +4369,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L16" s="68">
-        <v>1.2</v>
+      <c r="L16" s="65">
+        <v>0.35</v>
       </c>
       <c r="M16" s="27"/>
     </row>
@@ -4408,8 +4408,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L17" s="68">
-        <v>1.21</v>
+      <c r="L17" s="66">
+        <v>0.35</v>
       </c>
       <c r="M17" s="28"/>
     </row>
@@ -4447,8 +4447,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L18" s="68">
-        <v>1.1299999999999999</v>
+      <c r="L18" s="65">
+        <v>0.35</v>
       </c>
       <c r="M18" s="27"/>
     </row>
@@ -4486,8 +4486,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L19" s="68">
-        <v>2.8185000000000002</v>
+      <c r="L19" s="66">
+        <v>0.65</v>
       </c>
       <c r="M19" s="28"/>
     </row>
@@ -4525,8 +4525,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L20" s="68">
-        <v>1.395</v>
+      <c r="L20" s="65">
+        <v>0.25</v>
       </c>
       <c r="M20" s="27"/>
     </row>
@@ -4564,8 +4564,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L21" s="68">
-        <v>1.7045999999999999</v>
+      <c r="L21" s="66">
+        <v>0.3</v>
       </c>
       <c r="M21" s="28"/>
     </row>
@@ -4603,8 +4603,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L22" s="68">
-        <v>1.0049999999999999</v>
+      <c r="L22" s="65">
+        <v>0.3</v>
       </c>
       <c r="M22" s="27"/>
     </row>
@@ -4642,8 +4642,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L23" s="68">
-        <v>1.4419999999999999</v>
+      <c r="L23" s="66">
+        <v>0.4</v>
       </c>
       <c r="M23" s="28"/>
     </row>
@@ -4681,8 +4681,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L24" s="68">
-        <v>1.1679999999999999</v>
+      <c r="L24" s="65">
+        <v>0.48</v>
       </c>
       <c r="M24" s="27"/>
     </row>
@@ -4720,8 +4720,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L25" s="68">
-        <v>1.4550000000000001</v>
+      <c r="L25" s="66">
+        <v>0.52</v>
       </c>
       <c r="M25" s="28"/>
     </row>
@@ -4759,8 +4759,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L26" s="68">
-        <v>1.2825</v>
+      <c r="L26" s="65">
+        <v>2.3199999999999998</v>
       </c>
       <c r="M26" s="27"/>
     </row>
@@ -4798,8 +4798,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L27" s="68">
-        <v>2.2789999999999999</v>
+      <c r="L27" s="65">
+        <v>3.8</v>
       </c>
       <c r="M27" s="28"/>
     </row>
@@ -4837,8 +4837,8 @@
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="L28" s="68">
-        <v>1.6419999999999999</v>
+      <c r="L28" s="65">
+        <v>1.2</v>
       </c>
       <c r="M28" s="27"/>
     </row>
@@ -4876,8 +4876,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L29" s="68">
-        <v>1.5049999999999999</v>
+      <c r="L29" s="65">
+        <v>0.35</v>
       </c>
       <c r="M29" s="28"/>
     </row>
@@ -4915,8 +4915,8 @@
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="L30" s="68">
-        <v>1.2</v>
+      <c r="L30" s="65">
+        <v>0.65</v>
       </c>
       <c r="M30" s="27"/>
     </row>
@@ -4954,8 +4954,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L31" s="68">
-        <v>1.35</v>
+      <c r="L31" s="65">
+        <v>0.42</v>
       </c>
       <c r="M31" s="28"/>
     </row>
@@ -4993,8 +4993,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L32" s="68">
-        <v>1.3180000000000001</v>
+      <c r="L32" s="65">
+        <v>0.4</v>
       </c>
       <c r="M32" s="27"/>
     </row>
@@ -5032,8 +5032,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L33" s="68">
-        <v>2.4749999999999996</v>
+      <c r="L33" s="65">
+        <v>3.76</v>
       </c>
       <c r="M33" s="28"/>
     </row>
@@ -5071,8 +5071,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L34" s="68">
-        <v>1.3420000000000001</v>
+      <c r="L34" s="65">
+        <v>0.7</v>
       </c>
       <c r="M34" s="27"/>
     </row>
@@ -5110,8 +5110,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L35" s="68">
-        <v>1.294</v>
+      <c r="L35" s="65">
+        <v>0.48</v>
       </c>
       <c r="M35" s="28"/>
     </row>
@@ -5149,8 +5149,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L36" s="68">
-        <v>1.165</v>
+      <c r="L36" s="65">
+        <v>0.9</v>
       </c>
       <c r="M36" s="27"/>
     </row>
@@ -5188,8 +5188,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L37" s="68">
-        <v>1.18</v>
+      <c r="L37" s="65">
+        <v>0.75</v>
       </c>
       <c r="M37" s="28"/>
     </row>
@@ -5227,8 +5227,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L38" s="68">
-        <v>1.252</v>
+      <c r="L38" s="65">
+        <v>0.56000000000000005</v>
       </c>
       <c r="M38" s="27"/>
     </row>
@@ -5266,8 +5266,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L39" s="68">
-        <v>1.3220000000000001</v>
+      <c r="L39" s="65">
+        <v>0.67</v>
       </c>
       <c r="M39" s="28"/>
     </row>
@@ -5305,8 +5305,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L40" s="68">
-        <v>1.1600000000000001</v>
+      <c r="L40" s="65">
+        <v>0.38</v>
       </c>
       <c r="M40" s="27"/>
     </row>
@@ -5344,8 +5344,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L41" s="68">
-        <v>1.3460000000000001</v>
+      <c r="L41" s="65">
+        <v>0.78</v>
       </c>
       <c r="M41" s="28"/>
     </row>
@@ -5381,8 +5381,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L42" s="68">
-        <v>0.82</v>
+      <c r="L42" s="65">
+        <v>0.69</v>
       </c>
       <c r="M42" s="27"/>
     </row>
@@ -5420,8 +5420,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L43" s="68">
-        <v>0.87</v>
+      <c r="L43" s="65">
+        <v>0.6</v>
       </c>
       <c r="M43" s="28"/>
     </row>
@@ -5459,8 +5459,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L44" s="68">
-        <v>1.294</v>
+      <c r="L44" s="65">
+        <v>0.7</v>
       </c>
       <c r="M44" s="27"/>
     </row>
@@ -5498,8 +5498,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L45" s="68">
-        <v>1.248</v>
+      <c r="L45" s="65">
+        <v>0.45</v>
       </c>
       <c r="M45" s="28"/>
     </row>
@@ -5537,8 +5537,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L46" s="68">
-        <v>1.3540000000000001</v>
+      <c r="L46" s="65">
+        <v>0.5</v>
       </c>
       <c r="M46" s="27"/>
     </row>
@@ -5576,8 +5576,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L47" s="68">
-        <v>1.306</v>
+      <c r="L47" s="65">
+        <v>0.47</v>
       </c>
       <c r="M47" s="28"/>
     </row>
@@ -5615,8 +5615,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L48" s="68">
-        <v>1.3979999999999999</v>
+      <c r="L48" s="65">
+        <v>0.6</v>
       </c>
       <c r="M48" s="27"/>
     </row>
@@ -5654,8 +5654,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L49" s="68">
-        <v>1.266</v>
+      <c r="L49" s="65">
+        <v>0.8</v>
       </c>
       <c r="M49" s="28"/>
     </row>
@@ -5693,8 +5693,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L50" s="68">
-        <v>1.3380000000000001</v>
+      <c r="L50" s="65">
+        <v>0.45</v>
       </c>
       <c r="M50" s="27"/>
     </row>
@@ -5732,8 +5732,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L51" s="68">
-        <v>0.94</v>
+      <c r="L51" s="65">
+        <v>0.37</v>
       </c>
       <c r="M51" s="28"/>
     </row>
@@ -5771,8 +5771,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L52" s="68">
-        <v>1.522</v>
+      <c r="L52" s="65">
+        <v>0.4</v>
       </c>
       <c r="M52" s="27"/>
     </row>
@@ -5810,8 +5810,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L53" s="68">
-        <v>1.1839999999999999</v>
+      <c r="L53" s="65">
+        <v>0.33</v>
       </c>
       <c r="M53" s="28"/>
     </row>
@@ -5849,8 +5849,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L54" s="68">
-        <v>1.3740000000000001</v>
+      <c r="L54" s="65">
+        <v>0.3</v>
       </c>
       <c r="M54" s="27"/>
     </row>
@@ -5888,8 +5888,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L55" s="68">
-        <v>1.254</v>
+      <c r="L55" s="65">
+        <v>0.25</v>
       </c>
       <c r="M55" s="28"/>
     </row>
@@ -5927,8 +5927,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L56" s="68">
-        <v>1.224</v>
+      <c r="L56" s="65">
+        <v>0.44</v>
       </c>
       <c r="M56" s="27"/>
     </row>
@@ -5966,8 +5966,8 @@
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="L57" s="68">
-        <v>1.47</v>
+      <c r="L57" s="65">
+        <v>0.13</v>
       </c>
       <c r="M57" s="28"/>
     </row>
@@ -6005,8 +6005,8 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L58" s="68">
-        <v>1.258</v>
+      <c r="L58" s="65">
+        <v>0.45</v>
       </c>
       <c r="M58" s="27"/>
     </row>
@@ -6044,7 +6044,7 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="L59" s="68" t="s">
+      <c r="L59" s="65" t="s">
         <v>236</v>
       </c>
       <c r="M59" s="28"/>
@@ -6083,8 +6083,8 @@
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="L60" s="68">
-        <v>11.092000000000001</v>
+      <c r="L60" s="65">
+        <v>15.7</v>
       </c>
       <c r="M60" s="28"/>
       <c r="Q60" s="45"/>
@@ -6123,8 +6123,8 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="L61" s="68">
-        <v>1.889</v>
+      <c r="L61" s="65">
+        <v>5.4</v>
       </c>
       <c r="M61" s="28"/>
       <c r="Q61" s="45"/>
@@ -6137,27 +6137,27 @@
       <c r="F62" s="62"/>
       <c r="G62" s="63"/>
       <c r="H62" s="62"/>
-      <c r="I62" s="72" t="s">
+      <c r="I62" s="76" t="s">
         <v>259</v>
       </c>
-      <c r="J62" s="73"/>
-      <c r="K62" s="73"/>
-      <c r="L62" s="74">
+      <c r="J62" s="77"/>
+      <c r="K62" s="77"/>
+      <c r="L62" s="69">
         <f>SUM(L10:L61)</f>
-        <v>79.136599999999973</v>
+        <v>55.999999999999993</v>
       </c>
       <c r="M62" s="63"/>
       <c r="Q62" s="45"/>
     </row>
     <row r="63" spans="1:17" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I63" s="72" t="s">
+      <c r="I63" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="J63" s="73"/>
-      <c r="K63" s="73"/>
-      <c r="L63" s="75">
+      <c r="J63" s="77"/>
+      <c r="K63" s="77"/>
+      <c r="L63" s="70">
         <f>L62/2</f>
-        <v>39.568299999999986</v>
+        <v>27.999999999999996</v>
       </c>
     </row>
   </sheetData>
@@ -6200,11 +6200,11 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="65"/>
-      <c r="J1" s="65"/>
-      <c r="K1" s="65"/>
-      <c r="L1" s="65"/>
-      <c r="M1" s="65"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -6242,7 +6242,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="66"/>
+      <c r="M3" s="74"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -6261,7 +6261,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="46"/>
       <c r="L4" s="46"/>
-      <c r="M4" s="67"/>
+      <c r="M4" s="75"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -6280,7 +6280,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="46"/>
       <c r="L5" s="46"/>
-      <c r="M5" s="67"/>
+      <c r="M5" s="75"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -6295,7 +6295,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="46"/>
       <c r="L6" s="46"/>
-      <c r="M6" s="67"/>
+      <c r="M6" s="75"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -6310,7 +6310,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="67"/>
+      <c r="M7" s="75"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -6325,7 +6325,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="67"/>
+      <c r="M8" s="75"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -6400,8 +6400,8 @@
         <f>J10*5</f>
         <v>20</v>
       </c>
-      <c r="L10" s="68">
-        <v>1.52</v>
+      <c r="L10" s="65">
+        <v>0.88</v>
       </c>
       <c r="M10" s="27"/>
     </row>
@@ -6439,8 +6439,8 @@
         <f t="shared" ref="K11" si="1">J11*5</f>
         <v>20</v>
       </c>
-      <c r="L11" s="69">
-        <v>2.0760000000000001</v>
+      <c r="L11" s="66">
+        <v>0.78</v>
       </c>
       <c r="M11" s="28"/>
     </row>
@@ -6478,8 +6478,8 @@
         <f>J12*5</f>
         <v>5</v>
       </c>
-      <c r="L12" s="68">
-        <v>1.3450000000000002</v>
+      <c r="L12" s="65">
+        <v>0.65</v>
       </c>
       <c r="M12" s="27"/>
     </row>
@@ -6517,8 +6517,8 @@
         <f t="shared" ref="K13" si="2">J13*5</f>
         <v>5</v>
       </c>
-      <c r="L13" s="69">
-        <v>1.22</v>
+      <c r="L13" s="66">
+        <v>0.7</v>
       </c>
       <c r="M13" s="28"/>
     </row>
@@ -6556,8 +6556,8 @@
         <f>J14*5</f>
         <v>5</v>
       </c>
-      <c r="L14" s="68">
-        <v>1.3540000000000001</v>
+      <c r="L14" s="65">
+        <v>0.69</v>
       </c>
       <c r="M14" s="27"/>
     </row>
@@ -6595,8 +6595,8 @@
         <f t="shared" ref="K15" si="3">J15*5</f>
         <v>10</v>
       </c>
-      <c r="L15" s="69">
-        <v>1.4780000000000002</v>
+      <c r="L15" s="66">
+        <v>4.7</v>
       </c>
       <c r="M15" s="28"/>
     </row>
@@ -6634,8 +6634,8 @@
         <f>J16*5</f>
         <v>5</v>
       </c>
-      <c r="L16" s="68">
-        <v>1.37</v>
+      <c r="L16" s="65">
+        <v>0.7</v>
       </c>
       <c r="M16" s="27"/>
     </row>
@@ -6673,8 +6673,8 @@
         <f t="shared" ref="K17" si="4">J17*5</f>
         <v>5</v>
       </c>
-      <c r="L17" s="69">
-        <v>1.38</v>
+      <c r="L17" s="66">
+        <v>0.56000000000000005</v>
       </c>
       <c r="M17" s="28"/>
     </row>
@@ -6712,8 +6712,8 @@
         <f>J18*5</f>
         <v>5</v>
       </c>
-      <c r="L18" s="68">
-        <v>1.3</v>
+      <c r="L18" s="65">
+        <v>0.77</v>
       </c>
       <c r="M18" s="27"/>
     </row>
@@ -6751,8 +6751,8 @@
         <f t="shared" ref="K19" si="5">J19*5</f>
         <v>10</v>
       </c>
-      <c r="L19" s="69">
-        <v>5.4706999999999999</v>
+      <c r="L19" s="66">
+        <v>0.66</v>
       </c>
       <c r="M19" s="28"/>
     </row>
@@ -6790,8 +6790,8 @@
         <f>J20*5</f>
         <v>5</v>
       </c>
-      <c r="L20" s="68">
-        <v>1.5649999999999999</v>
+      <c r="L20" s="65">
+        <v>0.78</v>
       </c>
       <c r="M20" s="27"/>
     </row>
@@ -6829,8 +6829,8 @@
         <f t="shared" ref="K21" si="6">J21*5</f>
         <v>5</v>
       </c>
-      <c r="L21" s="69">
-        <v>2.8291999999999997</v>
+      <c r="L21" s="66">
+        <v>0.67500000000000004</v>
       </c>
       <c r="M21" s="28"/>
     </row>
@@ -6868,8 +6868,8 @@
         <f>J22*5</f>
         <v>5</v>
       </c>
-      <c r="L22" s="68">
-        <v>1.175</v>
+      <c r="L22" s="65">
+        <v>0.7</v>
       </c>
       <c r="M22" s="27"/>
     </row>
@@ -6907,8 +6907,8 @@
         <f t="shared" ref="K23" si="7">J23*5</f>
         <v>5</v>
       </c>
-      <c r="L23" s="69">
-        <v>1.6120000000000001</v>
+      <c r="L23" s="66">
+        <v>0.88</v>
       </c>
       <c r="M23" s="28"/>
     </row>
@@ -6946,8 +6946,8 @@
         <f>J24*5</f>
         <v>5</v>
       </c>
-      <c r="L24" s="68">
-        <v>1.756</v>
+      <c r="L24" s="65">
+        <v>0.8</v>
       </c>
       <c r="M24" s="27"/>
     </row>
@@ -6985,8 +6985,8 @@
         <f t="shared" ref="K25" si="8">J25*5</f>
         <v>5</v>
       </c>
-      <c r="L25" s="69">
-        <v>1.625</v>
+      <c r="L25" s="66">
+        <v>0.95</v>
       </c>
       <c r="M25" s="28"/>
     </row>
@@ -7024,8 +7024,8 @@
         <f>J26*5</f>
         <v>5</v>
       </c>
-      <c r="L26" s="68">
-        <v>1.9849999999999999</v>
+      <c r="L26" s="65">
+        <v>3.85</v>
       </c>
       <c r="M26" s="27"/>
     </row>
@@ -7063,7 +7063,7 @@
         <f t="shared" ref="K27" si="9">J27*5</f>
         <v>10</v>
       </c>
-      <c r="L27" s="69">
+      <c r="L27" s="66">
         <v>5.5070000000000006</v>
       </c>
       <c r="M27" s="28"/>
@@ -7102,8 +7102,8 @@
         <f>J28*5</f>
         <v>65</v>
       </c>
-      <c r="L28" s="68">
-        <v>2.7040000000000002</v>
+      <c r="L28" s="65">
+        <v>1.2</v>
       </c>
       <c r="M28" s="27"/>
     </row>
@@ -7141,8 +7141,8 @@
         <f t="shared" ref="K29" si="10">J29*5</f>
         <v>5</v>
       </c>
-      <c r="L29" s="69">
-        <v>1.675</v>
+      <c r="L29" s="66">
+        <v>0.76</v>
       </c>
       <c r="M29" s="28"/>
     </row>
@@ -7180,8 +7180,8 @@
         <f>J30*5</f>
         <v>20</v>
       </c>
-      <c r="L30" s="68">
-        <v>1.8199999999999998</v>
+      <c r="L30" s="65">
+        <v>1</v>
       </c>
       <c r="M30" s="27"/>
     </row>
@@ -7219,8 +7219,8 @@
         <f t="shared" ref="K31" si="11">J31*5</f>
         <v>10</v>
       </c>
-      <c r="L31" s="69">
-        <v>1.52</v>
+      <c r="L31" s="66">
+        <v>0.65</v>
       </c>
       <c r="M31" s="28"/>
     </row>
@@ -7258,8 +7258,8 @@
         <f>J32*5</f>
         <v>5</v>
       </c>
-      <c r="L32" s="68">
-        <v>1.488</v>
+      <c r="L32" s="65">
+        <v>0.75</v>
       </c>
       <c r="M32" s="27"/>
     </row>
@@ -7294,7 +7294,7 @@
         <f t="shared" ref="K33:K34" si="12">J33*5</f>
         <v>5</v>
       </c>
-      <c r="L33" s="68">
+      <c r="L33" s="65">
         <v>4.37</v>
       </c>
       <c r="M33" s="28"/>
@@ -7333,8 +7333,8 @@
         <f t="shared" si="12"/>
         <v>10</v>
       </c>
-      <c r="L34" s="68">
-        <v>1.512</v>
+      <c r="L34" s="65">
+        <v>0.75</v>
       </c>
       <c r="M34" s="27"/>
     </row>
@@ -7372,8 +7372,8 @@
         <f>J35*5</f>
         <v>5</v>
       </c>
-      <c r="L35" s="68">
-        <v>1.464</v>
+      <c r="L35" s="65">
+        <v>0.66</v>
       </c>
       <c r="M35" s="28"/>
     </row>
@@ -7411,8 +7411,8 @@
         <f t="shared" ref="K36" si="13">J36*5</f>
         <v>10</v>
       </c>
-      <c r="L36" s="68">
-        <v>1.335</v>
+      <c r="L36" s="65">
+        <v>0.78</v>
       </c>
       <c r="M36" s="27"/>
     </row>
@@ -7450,8 +7450,8 @@
         <f>J37*5</f>
         <v>15</v>
       </c>
-      <c r="L37" s="68">
-        <v>1.7799999999999998</v>
+      <c r="L37" s="65">
+        <v>0.9</v>
       </c>
       <c r="M37" s="28"/>
     </row>
@@ -7489,8 +7489,8 @@
         <f t="shared" ref="K38" si="14">J38*5</f>
         <v>10</v>
       </c>
-      <c r="L38" s="68">
-        <v>1.4220000000000002</v>
+      <c r="L38" s="65">
+        <v>0.75</v>
       </c>
       <c r="M38" s="27"/>
     </row>
@@ -7528,8 +7528,8 @@
         <f>J39*5</f>
         <v>15</v>
       </c>
-      <c r="L39" s="68">
-        <v>1.492</v>
+      <c r="L39" s="65">
+        <v>0.85</v>
       </c>
       <c r="M39" s="28"/>
     </row>
@@ -7567,8 +7567,8 @@
         <f t="shared" ref="K40" si="15">J40*5</f>
         <v>10</v>
       </c>
-      <c r="L40" s="68">
-        <v>1.33</v>
+      <c r="L40" s="65">
+        <v>0.77</v>
       </c>
       <c r="M40" s="27"/>
     </row>
@@ -7606,8 +7606,8 @@
         <f>J41*5</f>
         <v>15</v>
       </c>
-      <c r="L41" s="68">
-        <v>1.516</v>
+      <c r="L41" s="65">
+        <v>0.98</v>
       </c>
       <c r="M41" s="28"/>
     </row>
@@ -7643,8 +7643,8 @@
         <f t="shared" ref="K42" si="16">J42*5</f>
         <v>15</v>
       </c>
-      <c r="L42" s="68">
-        <v>0.99</v>
+      <c r="L42" s="65">
+        <v>0.76300000000000001</v>
       </c>
       <c r="M42" s="27"/>
     </row>
@@ -7682,8 +7682,8 @@
         <f>J43*5</f>
         <v>10</v>
       </c>
-      <c r="L43" s="68">
-        <v>1.04</v>
+      <c r="L43" s="65">
+        <v>0.8</v>
       </c>
       <c r="M43" s="28"/>
     </row>
@@ -7721,8 +7721,8 @@
         <f t="shared" ref="K44" si="17">J44*5</f>
         <v>15</v>
       </c>
-      <c r="L44" s="68">
-        <v>1.464</v>
+      <c r="L44" s="65">
+        <v>0.9</v>
       </c>
       <c r="M44" s="27"/>
     </row>
@@ -7760,8 +7760,8 @@
         <f>J45*5</f>
         <v>10</v>
       </c>
-      <c r="L45" s="68">
-        <v>1.4180000000000001</v>
+      <c r="L45" s="65">
+        <v>0.7</v>
       </c>
       <c r="M45" s="28"/>
     </row>
@@ -7799,8 +7799,8 @@
         <f t="shared" ref="K46" si="18">J46*5</f>
         <v>15</v>
       </c>
-      <c r="L46" s="68">
-        <v>1.524</v>
+      <c r="L46" s="65">
+        <v>0.81</v>
       </c>
       <c r="M46" s="27"/>
     </row>
@@ -7838,8 +7838,8 @@
         <f>J47*5</f>
         <v>10</v>
       </c>
-      <c r="L47" s="68">
-        <v>1.476</v>
+      <c r="L47" s="65">
+        <v>0.75</v>
       </c>
       <c r="M47" s="28"/>
     </row>
@@ -7877,8 +7877,8 @@
         <f t="shared" ref="K48" si="19">J48*5</f>
         <v>10</v>
       </c>
-      <c r="L48" s="68">
-        <v>1.5680000000000001</v>
+      <c r="L48" s="65">
+        <v>0.88</v>
       </c>
       <c r="M48" s="27"/>
     </row>
@@ -7916,8 +7916,8 @@
         <f>J49*5</f>
         <v>15</v>
       </c>
-      <c r="L49" s="68">
-        <v>1.4359999999999999</v>
+      <c r="L49" s="65">
+        <v>0.96</v>
       </c>
       <c r="M49" s="28"/>
     </row>
@@ -7955,8 +7955,8 @@
         <f t="shared" ref="K50" si="20">J50*5</f>
         <v>5</v>
       </c>
-      <c r="L50" s="68">
-        <v>1.508</v>
+      <c r="L50" s="65">
+        <v>0.48</v>
       </c>
       <c r="M50" s="27"/>
     </row>
@@ -7994,8 +7994,8 @@
         <f>J51*5</f>
         <v>5</v>
       </c>
-      <c r="L51" s="68">
-        <v>1.1100000000000001</v>
+      <c r="L51" s="65">
+        <v>0.55000000000000004</v>
       </c>
       <c r="M51" s="28"/>
     </row>
@@ -8033,8 +8033,8 @@
         <f t="shared" ref="K52" si="21">J52*5</f>
         <v>5</v>
       </c>
-      <c r="L52" s="68">
-        <v>1.6920000000000002</v>
+      <c r="L52" s="65">
+        <v>0.88</v>
       </c>
       <c r="M52" s="27"/>
     </row>
@@ -8072,8 +8072,8 @@
         <f>J53*5</f>
         <v>5</v>
       </c>
-      <c r="L53" s="68">
-        <v>1.3540000000000001</v>
+      <c r="L53" s="65">
+        <v>0.42</v>
       </c>
       <c r="M53" s="28"/>
     </row>
@@ -8111,8 +8111,8 @@
         <f t="shared" ref="K54" si="22">J54*5</f>
         <v>5</v>
       </c>
-      <c r="L54" s="68">
-        <v>1.544</v>
+      <c r="L54" s="65">
+        <v>0.53</v>
       </c>
       <c r="M54" s="27"/>
       <c r="P54"/>
@@ -8151,8 +8151,8 @@
         <f>J55*5</f>
         <v>5</v>
       </c>
-      <c r="L55" s="68">
-        <v>1.4239999999999999</v>
+      <c r="L55" s="65">
+        <v>0.68</v>
       </c>
       <c r="M55" s="28"/>
     </row>
@@ -8190,8 +8190,8 @@
         <f t="shared" ref="K56:K57" si="23">J56*5</f>
         <v>5</v>
       </c>
-      <c r="L56" s="68">
-        <v>1.3940000000000001</v>
+      <c r="L56" s="65">
+        <v>0.74</v>
       </c>
       <c r="M56" s="27"/>
     </row>
@@ -8229,7 +8229,7 @@
         <f t="shared" si="23"/>
         <v>5</v>
       </c>
-      <c r="L57" s="69">
+      <c r="L57" s="66">
         <v>2.36</v>
       </c>
       <c r="M57" s="28"/>
@@ -8268,8 +8268,8 @@
         <f>J58*5</f>
         <v>10</v>
       </c>
-      <c r="L58" s="68">
-        <v>1.4279999999999999</v>
+      <c r="L58" s="65">
+        <v>0.88</v>
       </c>
       <c r="M58" s="27"/>
     </row>
@@ -8307,7 +8307,7 @@
         <f t="shared" ref="K59" si="24">J59*5</f>
         <v>10</v>
       </c>
-      <c r="L59" s="70" t="s">
+      <c r="L59" s="67" t="s">
         <v>236</v>
       </c>
       <c r="M59" s="28"/>
@@ -8346,8 +8346,8 @@
         <f>J60*5</f>
         <v>45</v>
       </c>
-      <c r="L60" s="68">
-        <v>22.756200000000003</v>
+      <c r="L60" s="65">
+        <v>29.5</v>
       </c>
       <c r="M60" s="28"/>
       <c r="R60" s="45"/>
@@ -8386,8 +8386,8 @@
         <f t="shared" ref="K61" si="25">J61*5</f>
         <v>15</v>
       </c>
-      <c r="L61" s="71">
-        <v>3.198</v>
+      <c r="L61" s="68">
+        <v>10.199999999999999</v>
       </c>
       <c r="M61" s="51"/>
       <c r="R61" s="45"/>
@@ -8400,27 +8400,27 @@
       <c r="F62" s="56"/>
       <c r="G62" s="57"/>
       <c r="H62" s="56"/>
-      <c r="I62" s="72" t="s">
+      <c r="I62" s="76" t="s">
         <v>259</v>
       </c>
-      <c r="J62" s="73"/>
-      <c r="K62" s="73"/>
-      <c r="L62" s="74">
+      <c r="J62" s="77"/>
+      <c r="K62" s="77"/>
+      <c r="L62" s="69">
         <f>SUM(L10:L61)</f>
-        <v>112.68010000000001</v>
+        <v>94.185000000000016</v>
       </c>
       <c r="M62" s="64"/>
       <c r="R62" s="45"/>
     </row>
     <row r="63" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I63" s="72" t="s">
+      <c r="I63" s="76" t="s">
         <v>260</v>
       </c>
-      <c r="J63" s="73"/>
-      <c r="K63" s="73"/>
-      <c r="L63" s="75">
+      <c r="J63" s="77"/>
+      <c r="K63" s="77"/>
+      <c r="L63" s="70">
         <f>L62/5</f>
-        <v>22.536020000000001</v>
+        <v>18.837000000000003</v>
       </c>
       <c r="R63" s="45"/>
     </row>

</xml_diff>

<commit_message>
#7 Item Type Added
</commit_message>
<xml_diff>
--- a/Design Files/Xponent-tech/BOM/Client-BOM-Xponent-tech.xlsx
+++ b/Design Files/Xponent-tech/BOM/Client-BOM-Xponent-tech.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="263">
   <si>
     <t>Component list</t>
   </si>
@@ -3185,7 +3185,9 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C42" s="40"/>
+      <c r="C42" s="42" t="s">
+        <v>10</v>
+      </c>
       <c r="D42" s="48" t="s">
         <v>44</v>
       </c>
@@ -5355,7 +5357,9 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C42" s="40"/>
+      <c r="C42" s="42" t="s">
+        <v>10</v>
+      </c>
       <c r="D42" s="48" t="s">
         <v>44</v>
       </c>
@@ -7617,7 +7621,9 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C42" s="40"/>
+      <c r="C42" s="42" t="s">
+        <v>10</v>
+      </c>
       <c r="D42" s="48" t="s">
         <v>44</v>
       </c>

</xml_diff>